<commit_message>
Scorecard: 40/40/20 trailing/forward/absolute valuation blend
- Add forward P/E (analyst FY+1 EPS) and forward P/FCF (FCF margin × fwd rev)
  as second 40% component of P/E and P/FCF scoring
- Absolute valuation anchor (lookup table) weighted at 20%
- Bank PE absolute score capped at 6.0 to limit 2× weight amplification
- Pass analyst_ests to build_scorecard() in server.py and local_rerun.py;
  move analyst_ests fetch before scorecard call in server.py
- Bank ROE/NIM scoring, NCO rate moat/mgmt indicators, score normalisation
  to 0-10 scale, dashboard rescaling — all from this session

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/static/excel/ADBE_model.xlsx
+++ b/static/excel/ADBE_model.xlsx
@@ -7339,11 +7339,11 @@
         </is>
       </c>
       <c r="B5" s="43" t="n">
-        <v>95799.442</v>
+        <v>100079.92</v>
       </c>
       <c r="C5" s="44" t="inlineStr">
         <is>
-          <t>FMP marketCap  |  price $237.01</t>
+          <t>FMP marketCap  |  price $247.6</t>
         </is>
       </c>
     </row>
@@ -7425,11 +7425,11 @@
         </is>
       </c>
       <c r="B12" s="46" t="n">
-        <v>0.0446</v>
+        <v>0.0447</v>
       </c>
       <c r="C12" s="44" t="inlineStr">
         <is>
-          <t>FRED series DGS10  |  latest: 2026-05-13</t>
+          <t>FRED series DGS10  |  latest: 2026-05-14</t>
         </is>
       </c>
     </row>
@@ -7440,7 +7440,7 @@
         </is>
       </c>
       <c r="B13" s="48" t="n">
-        <v>0.0446</v>
+        <v>0.0447</v>
       </c>
       <c r="C13" s="49" t="inlineStr">
         <is>
@@ -7493,7 +7493,7 @@
     <row r="18">
       <c r="A18" s="17" t="inlineStr">
         <is>
-          <t>Damodaran industry unlevered  (Software - Infrastructure)</t>
+          <t>Damodaran industry unlevered  (Software - Application)</t>
         </is>
       </c>
       <c r="B18" s="50" t="n">
@@ -7512,7 +7512,7 @@
         </is>
       </c>
       <c r="B19" s="50" t="n">
-        <v>1.137</v>
+        <v>1.135</v>
       </c>
       <c r="C19" s="44">
         <f> unlevered × (1 + (1 − t) × D/E)</f>
@@ -7541,7 +7541,7 @@
         </is>
       </c>
       <c r="B21" s="51" t="n">
-        <v>1.243</v>
+        <v>1.242</v>
       </c>
       <c r="C21" s="49" t="inlineStr">
         <is>
@@ -7715,11 +7715,11 @@
         </is>
       </c>
       <c r="B36" s="46" t="n">
-        <v>0.05</v>
+        <v>0.0501</v>
       </c>
       <c r="C36" s="44" t="inlineStr">
         <is>
-          <t>Rf 4.46% + spread 0.54%</t>
+          <t>Rf 4.47% + spread 0.54%</t>
         </is>
       </c>
     </row>
@@ -7745,7 +7745,7 @@
         </is>
       </c>
       <c r="B38" s="48" t="n">
-        <v>0.0472</v>
+        <v>0.0473</v>
       </c>
       <c r="C38" s="49" t="inlineStr">
         <is>
@@ -9964,7 +9964,7 @@
         </is>
       </c>
       <c r="B61" s="112" t="n">
-        <v>237.01</v>
+        <v>247.6</v>
       </c>
       <c r="C61" s="104" t="n"/>
       <c r="D61" s="104" t="n"/>
@@ -10064,7 +10064,7 @@
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="114" t="inlineStr">
         <is>
-          <t>JS SCORECARD — ADBE  |  Master Prompt v2  |  15 May 2026  |  Sector bucket: Tech Growth</t>
+          <t>JS SCORECARD — ADBE  |  Master Prompt v2  |  16 May 2026  |  Sector bucket: Tech Growth</t>
         </is>
       </c>
     </row>
@@ -10264,7 +10264,7 @@
       </c>
       <c r="D11" s="130" t="inlineStr">
         <is>
-          <t>ROIC trend +22.7% ✓ (≥-2pp)  |  GM maintained +0.9% ✓  |  Op margin +2.0% ✓ (≥-2pp)  |  Capital returns MOD-LOW ✗  |  Share count -2.8%/yr ✓ (net buyback)  |  Goodwill/Equity 111% ✗ (&lt;40%)  [4/6 indicators positive — proxy score]</t>
+          <t>ROIC trend +22.7% ✓ (&gt;=-2pp)  |  GM maintained +0.9% ✓  |  Op margin +2.0% ✓ (≥-2pp)  |  Capital returns MOD-LOW ✗  |  Share count -2.8%/yr ✓ (net buyback)  |  Goodwill/Equity 111% ✗ (&lt;40%)  [4/6 indicators positive — proxy score]</t>
         </is>
       </c>
       <c r="E11" s="131" t="inlineStr">
@@ -10281,7 +10281,7 @@
       </c>
       <c r="H11" s="134" t="inlineStr">
         <is>
-          <t>ROIC trend +22.7% ✓ (≥-2pp)  |  GM maintained +0.9% ✓  |  Op margin +2.0% ✓ (≥-2pp)  |  Capital returns MOD-LOW ✗  |  Share count -2.8%/yr ✓ (net buyback)  |  Goodwill/Equity 111% ✗ (&lt;40%)  [4/6 indicators positive — proxy score]</t>
+          <t>ROIC trend +22.7% ✓ (&gt;=-2pp)  |  GM maintained +0.9% ✓  |  Op margin +2.0% ✓ (≥-2pp)  |  Capital returns MOD-LOW ✗  |  Share count -2.8%/yr ✓ (net buyback)  |  Goodwill/Equity 111% ✗ (&lt;40%)  [4/6 indicators positive — proxy score]</t>
         </is>
       </c>
     </row>
@@ -10618,7 +10618,7 @@
       </c>
       <c r="D23" s="130" t="inlineStr">
         <is>
-          <t>Current 13.8x  |  5yr avg 29.6x  |  Sector median 51.6x  |  DCF-implied 15.8x  [-13% vs benchmark]</t>
+          <t>Current 13.8x  |  5yr avg 29.6x  |  Sector median 51.6x  |  DCF-implied 15.7x  [-12% vs benchmark]</t>
         </is>
       </c>
       <c r="E23" s="136" t="inlineStr">
@@ -10627,7 +10627,7 @@
         </is>
       </c>
       <c r="F23" s="132" t="n">
-        <v>8.9</v>
+        <v>8.82</v>
       </c>
       <c r="G23" s="133">
         <f>IF(F23="",0,C23*F23*10)</f>
@@ -10635,7 +10635,7 @@
       </c>
       <c r="H23" s="134" t="inlineStr">
         <is>
-          <t>Current 13.8x  |  5yr avg 29.6x  |  Sector median 51.6x  |  DCF-implied 15.8x  [-13% vs benchmark]</t>
+          <t>Current 13.8x  |  5yr avg 29.6x  |  Sector median 51.6x  |  DCF-implied 15.7x  [-12% vs benchmark]</t>
         </is>
       </c>
     </row>

</xml_diff>